<commit_message>
Add hero-banner block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (7):
- blocks/hero-banner/hero-banner.css
- tools/importer/import-homepage.bundle.js
- tools/importer/import-homepage.js
- tools/importer/page-templates.json
- tools/importer/parsers/hero-banner.js
- tools/importer/reports/import-homepage.report.xlsx
- tools/importer/reports/index.report.json
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -40,7 +40,7 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["hero-banner","cards-icon","cards-promo","carousel-industry","cards-story","form","accordion-links"]</t>
+    <t>["hero-banner","hero-banner","hero-banner","cards-icon","cards-icon","cards-promo","columns-feature","columns-feature","carousel-industry","cards-story","form","accordion-links"]</t>
   </si>
   <si>
     <t>index</t>
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-03-06T03:51:11.034Z</t>
+    <t>2026-03-06T04:07:17.031Z</t>
   </si>
   <si>
     <t>AT&amp;T Business – Fiber Internet, Wireless, Phone, IoT, 5G Solutions</t>

</xml_diff>